<commit_message>
UPDATE 03 09 2026
</commit_message>
<xml_diff>
--- a/data/empresas/Pacifico Cable SpA/Estado de Flujos de Efectivo.xlsx
+++ b/data/empresas/Pacifico Cable SpA/Estado de Flujos de Efectivo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Mundo\Programa de informes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{282A75AF-61CD-4829-BD56-4B556B26D45E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71591B56-61BB-4235-817D-EA5DC49FCA91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,16 +16,40 @@
     <sheet name="Flujo_Efectivo" sheetId="1" r:id="rId1"/>
     <sheet name="_CONFIG_" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>Nota</t>
   </si>
   <si>
+    <t>31-12-2025
+M$</t>
+  </si>
+  <si>
+    <t>31-12-2024
+M$</t>
+  </si>
+  <si>
+    <t>Flujos de efectivo procedentes de (utilizados en) actividades de operación</t>
+  </si>
+  <si>
     <t>Cobros procedentes de las ventas de bienes y prestación de servicios</t>
   </si>
   <si>
@@ -111,16 +135,13 @@
   </si>
   <si>
     <t>version</t>
-  </si>
-  <si>
-    <t>M$</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -132,14 +153,6 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -173,7 +186,7 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="double">
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -182,21 +195,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -500,7 +508,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D25"/>
+  <dimension ref="A2:D34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="80" customWidth="1"/>
@@ -508,143 +516,193 @@
     <col min="3" max="4" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C1" s="2">
-        <v>46387</v>
-      </c>
-      <c r="D1" s="2">
-        <v>46022</v>
-      </c>
-    </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>2</v>
+      <c r="A4" s="3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
-        <v>8</v>
+      <c r="A10" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>9</v>
-      </c>
+      <c r="A11" s="4"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="A12" s="5" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="3" t="s">
+      <c r="B12" s="5"/>
+      <c r="C12" s="5">
+        <f>SUM(C5:C11)</f>
+        <v>0</v>
+      </c>
+      <c r="D12" s="5">
+        <f>SUM(D5:D11)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
         <v>11</v>
-      </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="4" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="4"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="5" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+      <c r="B18" s="5"/>
+      <c r="C18" s="5">
+        <f>SUM(C15:C17)</f>
+        <v>0</v>
+      </c>
+      <c r="D18" s="5">
+        <f>SUM(D15:D17)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="5" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="4"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="5" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="6" t="s">
+      <c r="B26" s="5"/>
+      <c r="C26" s="5">
+        <f>SUM(C21:C25)</f>
+        <v>0</v>
+      </c>
+      <c r="D26" s="5">
+        <f>SUM(D21:D25)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
         <v>21</v>
       </c>
-      <c r="B24" s="6"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-    </row>
-    <row r="25" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>22</v>
+      </c>
+      <c r="C30">
+        <f>+C26+C18+C12</f>
+        <v>0</v>
+      </c>
+      <c r="D30">
+        <f>+D26+D18+D12</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>23</v>
+      </c>
+      <c r="C32">
+        <f>+D34</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B34" s="5"/>
+      <c r="C34" s="5">
+        <f>+C32+C30+C28</f>
+        <v>0</v>
+      </c>
+      <c r="D34" s="5">
+        <f>+D32+D30</f>
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -657,15 +715,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B2">
         <v>2</v>
@@ -673,7 +731,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B3">
         <v>2</v>
@@ -681,7 +739,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -689,7 +747,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B5">
         <v>6</v>
@@ -697,7 +755,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B6">
         <v>5</v>
@@ -705,7 +763,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B7">
         <v>1</v>

</xml_diff>